<commit_message>
Improve PDF-backed template coverage and material extraction
</commit_message>
<xml_diff>
--- a/templates/approved/2. Протоколы.xlsx
+++ b/templates/approved/2. Протоколы.xlsx
@@ -5034,17 +5034,17 @@
         <v>358</v>
       </c>
       <c r="B23" s="115" t="str">
-        <f>CONCATENATE(B2,",",B3)</f>
+        <f>IF(AND(B2="",B3=""),"",CONCATENATE(IF(B2="","",B2),",",IF(B3="","",B3)))</f>
       </c>
       <c r="C23" s="115" t="str">
-        <f>CONCATENATE(C2,",",C3)</f>
+        <f>IF(AND(C2="",C3=""),"",CONCATENATE(IF(C2="","",C2),",",IF(C3="","",C3)))</f>
       </c>
       <c r="D23" s="116"/>
       <c r="F23" s="117" t="str">
-        <f>CONCATENATE(F8," ",F1,"-",F10," .",F9)</f>
+        <f>IF(AND(F8="",F1="",F10="",F9=""),"",CONCATENATE(IF(F8="","",F8)," ",IF(F1="","",F1),"-",IF(F10="","",F10)," .",IF(F9="","",F9)))</f>
       </c>
       <c r="G23" s="117" t="str">
-        <f>CONCATENATE(G8," ",F1,"-",G10," .",G9)</f>
+        <f>IF(AND(G8="",F1="",G10="",G9=""),"",CONCATENATE(IF(G8="","",G8)," ",IF(F1="","",F1),"-",IF(G10="","",G10)," .",IF(G9="","",G9)))</f>
       </c>
     </row>
     <row r="24" spans="1:7" ht="105" x14ac:dyDescent="0.25">
@@ -5052,82 +5052,82 @@
         <v>358</v>
       </c>
       <c r="B24" s="115" t="str">
-        <f>CONCATENATE(B1,",",B2,",",B3)</f>
+        <f>IF(AND(B1="",B2="",B3=""),"",CONCATENATE(IF(B1="","",B1),",",IF(B2="","",B2),",",IF(B3="","",B3)))</f>
       </c>
       <c r="C24" s="115" t="str">
-        <f>CONCATENATE(C1,",",C2,",",C3)</f>
+        <f>IF(AND(C1="",C2="",C3=""),"",CONCATENATE(IF(C1="","",C1),",",IF(C2="","",C2),",",IF(C3="","",C3)))</f>
       </c>
       <c r="D24" s="116"/>
       <c r="F24" s="117" t="str">
-        <f>CONCATENATE(F8," ",F1,"-",F10)</f>
+        <f>IF(AND(F8="",F1="",F10=""),"",CONCATENATE(IF(F8="","",F8)," ",IF(F1="","",F1),"-",IF(F10="","",F10)))</f>
       </c>
       <c r="G24" s="117" t="str">
-        <f>CONCATENATE(G8," ",F1,"-",G10)</f>
+        <f>IF(AND(G8="",F1="",G10=""),"",CONCATENATE(IF(G8="","",G8)," ",IF(F1="","",F1),"-",IF(G10="","",G10)))</f>
       </c>
     </row>
     <row r="25" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="B25" s="118" t="str">
-        <f>CONCATENATE(B8," ",B1,"-",B10,".",B9)</f>
+        <f>IF(AND(B8="",B1="",B10="",B9=""),"",CONCATENATE(IF(B8="","",B8)," ",IF(B1="","",B1),"-",IF(B10="","",B10),".",IF(B9="","",B9)))</f>
       </c>
       <c r="C25" s="118" t="str">
-        <f>CONCATENATE(C8," ",C1,"-",C10,".",C9)</f>
+        <f>IF(AND(C8="",C1="",C10="",C9=""),"",CONCATENATE(IF(C8="","",C8)," ",IF(C1="","",C1),"-",IF(C10="","",C10),".",IF(C9="","",C9)))</f>
       </c>
       <c r="D25" s="119"/>
       <c r="F25" s="117" t="str">
-        <f>CONCATENATE(F8," ",F1)</f>
+        <f>IF(AND(F8="",F1=""),"",CONCATENATE(IF(F8="","",F8)," ",IF(F1="","",F1)))</f>
       </c>
       <c r="G25" s="117" t="str">
-        <f>CONCATENATE(G8," ",F1)</f>
+        <f>IF(AND(G8="",F1=""),"",CONCATENATE(IF(G8="","",G8)," ",IF(F1="","",F1)))</f>
       </c>
     </row>
     <row r="26" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="B26" s="118" t="str">
-        <f>CONCATENATE(B8," ",B1)</f>
+        <f>IF(AND(B8="",B1=""),"",CONCATENATE(IF(B8="","",B8)," ",IF(B1="","",B1)))</f>
       </c>
       <c r="C26" s="118" t="str">
-        <f>CONCATENATE(C8," ",C1)</f>
+        <f>IF(AND(C8="",C1=""),"",CONCATENATE(IF(C8="","",C8)," ",IF(C1="","",C1)))</f>
       </c>
       <c r="D26" s="119"/>
       <c r="F26" s="54" t="str">
-        <f>CONCATENATE(F6," ",F1," ",F7)</f>
+        <f>IF(AND(F6="",F1="",F7=""),"",CONCATENATE(IF(F6="","",F6)," ",IF(F1="","",F1)," ",IF(F7="","",F7)))</f>
       </c>
       <c r="G26" s="54" t="str">
-        <f>CONCATENATE(G6," ",F1," ",G7)</f>
+        <f>IF(AND(G6="",F1="",G7=""),"",CONCATENATE(IF(G6="","",G6)," ",IF(F1="","",F1)," ",IF(G7="","",G7)))</f>
       </c>
     </row>
     <row r="27" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="B27" s="120" t="str">
-        <f>CONCATENATE(B18," ",B1,"-",B20,".",B19)</f>
+        <f>IF(AND(B18="",B1="",B20="",B19=""),"",CONCATENATE(IF(B18="","",B18)," ",IF(B1="","",B1),"-",IF(B20="","",B20),".",IF(B19="","",B19)))</f>
       </c>
       <c r="C27" s="120" t="str">
-        <f>CONCATENATE(C18," ",C1,"-",C20,".",C19)</f>
+        <f>IF(AND(C18="",C1="",C20="",C19=""),"",CONCATENATE(IF(C18="","",C18)," ",IF(C1="","",C1),"-",IF(C20="","",C20),".",IF(C19="","",C19)))</f>
       </c>
       <c r="D27" s="117"/>
       <c r="F27" s="121" t="str">
-        <f>CONCATENATE(F14," ",F1," ",F15)</f>
+        <f>IF(AND(F14="",F1="",F15=""),"",CONCATENATE(IF(F14="","",F14)," ",IF(F1="","",F1)," ",IF(F15="","",F15)))</f>
       </c>
       <c r="G27" s="121" t="str">
-        <f>CONCATENATE(G14," ",F1," ",G15)</f>
+        <f>IF(AND(G14="",F1="",G15=""),"",CONCATENATE(IF(G14="","",G14)," ",IF(F1="","",F1)," ",IF(G15="","",G15)))</f>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B28" s="120" t="str">
-        <f>CONCATENATE(B18," ",B1," ",B20)</f>
+        <f>IF(AND(B18="",B1="",B20=""),"",CONCATENATE(IF(B18="","",B18)," ",IF(B1="","",B1)," ",IF(B20="","",B20)))</f>
       </c>
       <c r="C28" s="120" t="str">
-        <f>CONCATENATE(C18," ",C1,"-",C20)</f>
+        <f>IF(AND(C18="",C1="",C20=""),"",CONCATENATE(IF(C18="","",C18)," ",IF(C1="","",C1),"-",IF(C20="","",C20)))</f>
       </c>
       <c r="D28" s="117"/>
       <c r="F28" s="54" t="str">
-        <f>CONCATENATE(F16," ",F1," ",F17)</f>
+        <f>IF(AND(F16="",F1="",F17=""),"",CONCATENATE(IF(F16="","",F16)," ",IF(F1="","",F1)," ",IF(F17="","",F17)))</f>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B29" s="122" t="str">
-        <f>CONCATENATE(B18," ",B1)</f>
+        <f>IF(AND(B18="",B1=""),"",CONCATENATE(IF(B18="","",B18)," ",IF(B1="","",B1)))</f>
       </c>
       <c r="C29" s="120" t="str">
-        <f>CONCATENATE(C18," ",C1)</f>
+        <f>IF(AND(C18="",C1=""),"",CONCATENATE(IF(C18="","",C18)," ",IF(C1="","",C1)))</f>
       </c>
       <c r="D29" s="117"/>
     </row>
@@ -5159,7 +5159,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -5168,7 +5168,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -5176,7 +5176,7 @@
     </row>
     <row r="2" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -5200,7 +5200,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -5231,7 +5231,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -5616,7 +5616,7 @@
         <v>274</v>
       </c>
       <c r="C24" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D24" s="3" t="s">
         <v>265</v>
@@ -5627,7 +5627,7 @@
         <v>275</v>
       </c>
       <c r="C25" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D25" s="3" t="s">
         <v>267</v>
@@ -5638,7 +5638,7 @@
         <v>276</v>
       </c>
       <c r="C26" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D26" s="3" t="s">
         <v>269</v>
@@ -5728,10 +5728,10 @@
         <v>45</v>
       </c>
       <c r="I32" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J32" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K32" s="291"/>
     </row>
@@ -5751,10 +5751,10 @@
       </c>
       <c r="H33" s="142"/>
       <c r="I33" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J33" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K33" s="293"/>
     </row>
@@ -5774,10 +5774,10 @@
       </c>
       <c r="H34" s="142"/>
       <c r="I34" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J34" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K34" s="293"/>
     </row>
@@ -5797,10 +5797,10 @@
       </c>
       <c r="H35" s="142"/>
       <c r="I35" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J35" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K35" s="293"/>
     </row>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
@@ -5896,7 +5896,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="140"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J44" s="247"/>
       <c r="K44" s="140"/>
@@ -5956,7 +5956,7 @@
       <c r="A48" s="245"/>
       <c r="B48" s="245"/>
       <c r="C48" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D48" s="247"/>
       <c r="E48" s="247"/>
@@ -5964,7 +5964,7 @@
       <c r="G48" s="6"/>
       <c r="H48" s="140"/>
       <c r="I48" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J48" s="247"/>
       <c r="K48" s="140"/>
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B51" s="245"/>
       <c r="C51" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D51" s="247"/>
       <c r="E51" s="247"/>
@@ -6017,7 +6017,7 @@
       <c r="G51" s="6"/>
       <c r="H51" s="140"/>
       <c r="I51" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J51" s="247"/>
       <c r="K51" s="140"/>
@@ -6127,7 +6127,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -6136,7 +6136,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -6144,7 +6144,7 @@
     </row>
     <row r="2" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -6153,7 +6153,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="260" t="str">
-        <f>CONCATENATE('Данные объект'!$B$17, " ",'Данные объект'!$B$18)</f>
+        <f>IF(AND('Данные объект'!$B$17="",'Данные объект'!$B$18=""),"",CONCATENATE(IF('Данные объект'!$B$17="","",'Данные объект'!$B$17), " ",IF('Данные объект'!$B$18="","",'Данные объект'!$B$18)))</f>
       </c>
       <c r="I2" s="260"/>
       <c r="J2" s="260"/>
@@ -6168,7 +6168,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -6199,7 +6199,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -6507,7 +6507,7 @@
         <v>270</v>
       </c>
       <c r="C28" s="393">
-        <f>'Данные объект'!B10</f>
+        <f>IF('Данные объект'!B10="","",'Данные объект'!B10)</f>
       </c>
       <c r="D28" s="3" t="s">
         <v>265</v>
@@ -6518,7 +6518,7 @@
         <v>271</v>
       </c>
       <c r="C29" s="393">
-        <f>'Данные объект'!B11</f>
+        <f>IF('Данные объект'!B11="","",'Данные объект'!B11)</f>
       </c>
       <c r="D29" s="3" t="s">
         <v>267</v>
@@ -6529,7 +6529,7 @@
         <v>272</v>
       </c>
       <c r="C30" s="393" t="str">
-        <f>'Данные объект'!B12</f>
+        <f>IF('Данные объект'!B12="","",'Данные объект'!B12)</f>
       </c>
       <c r="D30" s="3" t="s">
         <v>269</v>
@@ -6637,10 +6637,10 @@
         <v>45</v>
       </c>
       <c r="I37" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J37" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K37" s="291"/>
     </row>
@@ -6660,10 +6660,10 @@
       </c>
       <c r="H38" s="142"/>
       <c r="I38" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J38" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K38" s="293"/>
     </row>
@@ -6683,10 +6683,10 @@
       </c>
       <c r="H39" s="142"/>
       <c r="I39" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J39" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K39" s="293"/>
     </row>
@@ -6706,10 +6706,10 @@
       </c>
       <c r="H40" s="142"/>
       <c r="I40" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J40" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K40" s="293"/>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="B43" s="245"/>
       <c r="C43" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D43" s="247"/>
       <c r="E43" s="247"/>
@@ -6742,7 +6742,7 @@
       <c r="G43" s="6"/>
       <c r="H43" s="140"/>
       <c r="I43" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J43" s="247"/>
       <c r="K43" s="140"/>
@@ -6802,7 +6802,7 @@
       <c r="A47" s="245"/>
       <c r="B47" s="245"/>
       <c r="C47" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D47" s="247"/>
       <c r="E47" s="247"/>
@@ -6810,7 +6810,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="140"/>
       <c r="I47" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J47" s="247"/>
       <c r="K47" s="140"/>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="B50" s="245"/>
       <c r="C50" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D50" s="247"/>
       <c r="E50" s="247"/>
@@ -6863,7 +6863,7 @@
       <c r="G50" s="6"/>
       <c r="H50" s="140"/>
       <c r="I50" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J50" s="247"/>
       <c r="K50" s="140"/>
@@ -6995,7 +6995,7 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -7004,7 +7004,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -7012,7 +7012,7 @@
     </row>
     <row r="2" spans="1:16" s="3" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -7021,7 +7021,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="260" t="str">
-        <f>CONCATENATE('Данные объект'!$B$17, " ",'Данные объект'!$B$18)</f>
+        <f>IF(AND('Данные объект'!$B$17="",'Данные объект'!$B$18=""),"",CONCATENATE(IF('Данные объект'!$B$17="","",'Данные объект'!$B$17), " ",IF('Данные объект'!$B$18="","",'Данные объект'!$B$18)))</f>
       </c>
       <c r="I2" s="260"/>
       <c r="J2" s="260"/>
@@ -7036,7 +7036,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -7067,7 +7067,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -7422,7 +7422,7 @@
         <v>274</v>
       </c>
       <c r="C20" s="392">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D20" s="3" t="s">
         <v>265</v>
@@ -7433,7 +7433,7 @@
         <v>275</v>
       </c>
       <c r="C21" s="392">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D21" s="3" t="s">
         <v>267</v>
@@ -7444,7 +7444,7 @@
         <v>276</v>
       </c>
       <c r="C22" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D22" s="3" t="s">
         <v>269</v>
@@ -7557,10 +7557,10 @@
         <v>45</v>
       </c>
       <c r="I28" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J28" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K28" s="291"/>
     </row>
@@ -7580,10 +7580,10 @@
       </c>
       <c r="H29" s="142"/>
       <c r="I29" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J29" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K29" s="293"/>
     </row>
@@ -7603,10 +7603,10 @@
       </c>
       <c r="H30" s="142"/>
       <c r="I30" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J30" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K30" s="293"/>
     </row>
@@ -7626,10 +7626,10 @@
       </c>
       <c r="H31" s="142"/>
       <c r="I31" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J31" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K31" s="293"/>
     </row>
@@ -7684,7 +7684,7 @@
       </c>
       <c r="B36" s="245"/>
       <c r="C36" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D36" s="247"/>
       <c r="E36" s="247"/>
@@ -7692,7 +7692,7 @@
       <c r="G36" s="6"/>
       <c r="H36" s="140"/>
       <c r="I36" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J36" s="247"/>
       <c r="K36" s="140"/>
@@ -7752,7 +7752,7 @@
       <c r="A40" s="245"/>
       <c r="B40" s="245"/>
       <c r="C40" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D40" s="247"/>
       <c r="E40" s="247"/>
@@ -7760,7 +7760,7 @@
       <c r="G40" s="6"/>
       <c r="H40" s="140"/>
       <c r="I40" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J40" s="247"/>
       <c r="K40" s="140"/>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="B43" s="245"/>
       <c r="C43" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D43" s="247"/>
       <c r="E43" s="247"/>
@@ -7813,7 +7813,7 @@
       <c r="G43" s="6"/>
       <c r="H43" s="140"/>
       <c r="I43" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J43" s="247"/>
       <c r="K43" s="140"/>
@@ -7922,7 +7922,7 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -7931,7 +7931,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -7939,7 +7939,7 @@
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -7963,7 +7963,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -7994,7 +7994,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -8094,7 +8094,7 @@
     <row r="13" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="60"/>
       <c r="B13" s="320" t="str">
-        <f>H2</f>
+        <f>IF(H2="","",H2)</f>
       </c>
       <c r="C13" s="320"/>
       <c r="D13" s="320"/>
@@ -8197,7 +8197,7 @@
         <v>274</v>
       </c>
       <c r="C19" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D19" s="3" t="s">
         <v>265</v>
@@ -8208,7 +8208,7 @@
         <v>275</v>
       </c>
       <c r="C20" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D20" s="3" t="s">
         <v>267</v>
@@ -8219,7 +8219,7 @@
         <v>276</v>
       </c>
       <c r="C21" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D21" s="3" t="s">
         <v>269</v>
@@ -8327,10 +8327,10 @@
         <v>45</v>
       </c>
       <c r="I28" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J28" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K28" s="291"/>
     </row>
@@ -8350,10 +8350,10 @@
       </c>
       <c r="H29" s="142"/>
       <c r="I29" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J29" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K29" s="293"/>
     </row>
@@ -8373,10 +8373,10 @@
       </c>
       <c r="H30" s="142"/>
       <c r="I30" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J30" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K30" s="293"/>
     </row>
@@ -8396,10 +8396,10 @@
       </c>
       <c r="H31" s="142"/>
       <c r="I31" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J31" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K31" s="293"/>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="B37" s="245"/>
       <c r="C37" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D37" s="247"/>
       <c r="E37" s="247"/>
@@ -8447,7 +8447,7 @@
       <c r="G37" s="6"/>
       <c r="H37" s="140"/>
       <c r="I37" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J37" s="247"/>
       <c r="K37" s="140"/>
@@ -8507,7 +8507,7 @@
       <c r="A41" s="245"/>
       <c r="B41" s="245"/>
       <c r="C41" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D41" s="247"/>
       <c r="E41" s="247"/>
@@ -8515,7 +8515,7 @@
       <c r="G41" s="6"/>
       <c r="H41" s="140"/>
       <c r="I41" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J41" s="247"/>
       <c r="K41" s="140"/>
@@ -8560,7 +8560,7 @@
       </c>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
@@ -8568,7 +8568,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="140"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J44" s="247"/>
       <c r="K44" s="140"/>
@@ -8672,7 +8672,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -8681,7 +8681,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -8689,7 +8689,7 @@
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -8698,7 +8698,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="260" t="str">
-        <f>CONCATENATE('Данные объект'!$B$17, " ",'Данные объект'!$B$18)</f>
+        <f>IF(AND('Данные объект'!$B$17="",'Данные объект'!$B$18=""),"",CONCATENATE(IF('Данные объект'!$B$17="","",'Данные объект'!$B$17), " ",IF('Данные объект'!$B$18="","",'Данные объект'!$B$18)))</f>
       </c>
       <c r="I2" s="260"/>
       <c r="J2" s="260"/>
@@ -8713,7 +8713,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -8744,7 +8744,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -8864,7 +8864,7 @@
       <c r="F14" s="326"/>
       <c r="G14" s="326"/>
       <c r="H14" s="326" t="str">
-        <f t="shared" ref="H14:H17" si="0">$H$13</f>
+        <f t="shared" ref="H14:H17" si="0">IF($H$13="","",$H$13)</f>
       </c>
       <c r="I14" s="326"/>
       <c r="J14" s="324" t="s">
@@ -8949,7 +8949,7 @@
         <v>264</v>
       </c>
       <c r="C20" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D20" s="3" t="s">
         <v>265</v>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="B21" s="32"/>
       <c r="C21" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D21" s="3" t="s">
         <v>267</v>
@@ -8972,7 +8972,7 @@
         <v>268</v>
       </c>
       <c r="C22" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D22" s="3" t="s">
         <v>269</v>
@@ -9075,10 +9075,10 @@
         <v>45</v>
       </c>
       <c r="I28" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J28" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K28" s="291"/>
     </row>
@@ -9098,10 +9098,10 @@
       </c>
       <c r="H29" s="142"/>
       <c r="I29" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J29" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K29" s="293"/>
     </row>
@@ -9121,10 +9121,10 @@
       </c>
       <c r="H30" s="142"/>
       <c r="I30" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J30" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K30" s="293"/>
     </row>
@@ -9144,10 +9144,10 @@
       </c>
       <c r="H31" s="142"/>
       <c r="I31" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J31" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K31" s="293"/>
     </row>
@@ -9237,7 +9237,7 @@
       </c>
       <c r="B40" s="245"/>
       <c r="C40" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D40" s="247"/>
       <c r="E40" s="247"/>
@@ -9245,7 +9245,7 @@
       <c r="G40" s="6"/>
       <c r="H40" s="140"/>
       <c r="I40" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J40" s="247"/>
       <c r="K40" s="140"/>
@@ -9305,7 +9305,7 @@
       <c r="A44" s="245"/>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
@@ -9313,7 +9313,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="140"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J44" s="247"/>
       <c r="K44" s="140"/>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="B47" s="245"/>
       <c r="C47" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D47" s="247"/>
       <c r="E47" s="247"/>
@@ -9366,7 +9366,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="140"/>
       <c r="I47" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J47" s="247"/>
       <c r="K47" s="140"/>
@@ -9489,7 +9489,7 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -9498,7 +9498,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -9506,7 +9506,7 @@
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -9515,7 +9515,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="260" t="str">
-        <f>'Данные объект'!B18</f>
+        <f>IF('Данные объект'!B18="","",'Данные объект'!B18)</f>
       </c>
       <c r="I2" s="260"/>
       <c r="J2" s="260"/>
@@ -9530,7 +9530,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -9561,7 +9561,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -9718,7 +9718,7 @@
         <v>274</v>
       </c>
       <c r="C17" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D17" s="3" t="s">
         <v>265</v>
@@ -9729,7 +9729,7 @@
         <v>275</v>
       </c>
       <c r="C18" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D18" s="3" t="s">
         <v>267</v>
@@ -9740,7 +9740,7 @@
         <v>276</v>
       </c>
       <c r="C19" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D19" s="3" t="s">
         <v>269</v>
@@ -9843,10 +9843,10 @@
         <v>45</v>
       </c>
       <c r="I25" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J25" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K25" s="291"/>
     </row>
@@ -9866,10 +9866,10 @@
       </c>
       <c r="H26" s="142"/>
       <c r="I26" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J26" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K26" s="293"/>
     </row>
@@ -9889,10 +9889,10 @@
       </c>
       <c r="H27" s="142"/>
       <c r="I27" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J27" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K27" s="293"/>
     </row>
@@ -9912,10 +9912,10 @@
       </c>
       <c r="H28" s="142"/>
       <c r="I28" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J28" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K28" s="293"/>
     </row>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="B38" s="245"/>
       <c r="C38" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D38" s="247"/>
       <c r="E38" s="247"/>
@@ -9998,7 +9998,7 @@
       <c r="G38" s="6"/>
       <c r="H38" s="140"/>
       <c r="I38" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J38" s="247"/>
       <c r="K38" s="140"/>
@@ -10058,7 +10058,7 @@
       <c r="A42" s="245"/>
       <c r="B42" s="245"/>
       <c r="C42" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D42" s="247"/>
       <c r="E42" s="247"/>
@@ -10066,7 +10066,7 @@
       <c r="G42" s="6"/>
       <c r="H42" s="140"/>
       <c r="I42" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J42" s="247"/>
       <c r="K42" s="140"/>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="B45" s="245"/>
       <c r="C45" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D45" s="247"/>
       <c r="E45" s="247"/>
@@ -10119,7 +10119,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="140"/>
       <c r="I45" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J45" s="247"/>
       <c r="K45" s="140"/>
@@ -10224,7 +10224,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -10234,7 +10234,7 @@
         <v>11</v>
       </c>
       <c r="I1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="J1" s="259"/>
       <c r="K1" s="259"/>
@@ -10242,7 +10242,7 @@
     </row>
     <row r="2" spans="1:15" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -10252,7 +10252,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="260" t="str">
-        <f>'Данные объект'!B19</f>
+        <f>IF('Данные объект'!B19="","",'Данные объект'!B19)</f>
       </c>
       <c r="J2" s="260"/>
       <c r="K2" s="260"/>
@@ -10268,7 +10268,7 @@
         <v>13</v>
       </c>
       <c r="I3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="J3" s="261"/>
       <c r="K3" s="261"/>
@@ -10302,7 +10302,7 @@
       <c r="C6" s="250"/>
       <c r="D6" s="250"/>
       <c r="K6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="L6" s="263"/>
     </row>
@@ -10690,7 +10690,7 @@
         <v>274</v>
       </c>
       <c r="C25" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D25" s="3" t="s">
         <v>265</v>
@@ -10701,7 +10701,7 @@
         <v>275</v>
       </c>
       <c r="C26" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D26" s="3" t="s">
         <v>267</v>
@@ -10712,7 +10712,7 @@
         <v>276</v>
       </c>
       <c r="C27" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D27" s="3" t="s">
         <v>269</v>
@@ -10829,10 +10829,10 @@
         <v>45</v>
       </c>
       <c r="I34" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J34" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K34" s="291"/>
     </row>
@@ -10852,10 +10852,10 @@
       </c>
       <c r="H35" s="142"/>
       <c r="I35" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J35" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K35" s="293"/>
     </row>
@@ -10875,10 +10875,10 @@
       </c>
       <c r="H36" s="142"/>
       <c r="I36" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J36" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K36" s="293"/>
     </row>
@@ -10898,10 +10898,10 @@
       </c>
       <c r="H37" s="142"/>
       <c r="I37" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J37" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K37" s="293"/>
     </row>
@@ -10912,7 +10912,7 @@
       </c>
       <c r="B40" s="245"/>
       <c r="C40" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D40" s="247"/>
       <c r="E40" s="247"/>
@@ -10920,7 +10920,7 @@
       <c r="G40" s="6"/>
       <c r="H40" s="140"/>
       <c r="I40" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J40" s="247"/>
       <c r="K40" s="140"/>
@@ -10980,7 +10980,7 @@
       <c r="A44" s="245"/>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
@@ -10988,7 +10988,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="140"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J44" s="247"/>
       <c r="K44" s="140"/>
@@ -11033,7 +11033,7 @@
       </c>
       <c r="B47" s="245"/>
       <c r="C47" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D47" s="247"/>
       <c r="E47" s="247"/>
@@ -11041,7 +11041,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="140"/>
       <c r="I47" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J47" s="247"/>
       <c r="K47" s="140"/>
@@ -11242,7 +11242,7 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -11251,7 +11251,7 @@
         <v>11</v>
       </c>
       <c r="G1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="H1" s="259"/>
       <c r="I1" s="259"/>
@@ -11259,7 +11259,7 @@
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -11268,7 +11268,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="260" t="str">
-        <f>'Данные объект'!B17</f>
+        <f>IF('Данные объект'!B17="","",'Данные объект'!B17)</f>
       </c>
       <c r="H2" s="260"/>
       <c r="I2" s="260"/>
@@ -11283,7 +11283,7 @@
         <v>13</v>
       </c>
       <c r="G3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="H3" s="261"/>
       <c r="I3" s="261"/>
@@ -11314,7 +11314,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="I6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="J6" s="263"/>
     </row>
@@ -11588,7 +11588,7 @@
       </c>
       <c r="B22" s="245"/>
       <c r="C22" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D22" s="247"/>
       <c r="E22" s="247"/>
@@ -11596,7 +11596,7 @@
       <c r="G22" s="6"/>
       <c r="H22" s="140"/>
       <c r="I22" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J22" s="247"/>
       <c r="K22" s="140"/>
@@ -11656,7 +11656,7 @@
       <c r="A26" s="245"/>
       <c r="B26" s="245"/>
       <c r="C26" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D26" s="247"/>
       <c r="E26" s="247"/>
@@ -11664,7 +11664,7 @@
       <c r="G26" s="6"/>
       <c r="H26" s="140"/>
       <c r="I26" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J26" s="247"/>
       <c r="K26" s="140"/>
@@ -11709,7 +11709,7 @@
       </c>
       <c r="B29" s="245"/>
       <c r="C29" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D29" s="247"/>
       <c r="E29" s="247"/>
@@ -11717,7 +11717,7 @@
       <c r="G29" s="6"/>
       <c r="H29" s="140"/>
       <c r="I29" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J29" s="247"/>
       <c r="K29" s="140"/>
@@ -12038,7 +12038,7 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -12047,7 +12047,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -12055,7 +12055,7 @@
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -12064,7 +12064,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="260" t="str">
-        <f>'Данные объект'!B14</f>
+        <f>IF('Данные объект'!B14="","",'Данные объект'!B14)</f>
       </c>
       <c r="I2" s="260"/>
       <c r="J2" s="260"/>
@@ -12079,7 +12079,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -12110,7 +12110,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -12139,7 +12139,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="360" t="str">
-        <f>'Данные объект'!B14</f>
+        <f>IF('Данные объект'!B14="","",'Данные объект'!B14)</f>
       </c>
       <c r="B13" s="360"/>
       <c r="C13" s="360"/>
@@ -12153,7 +12153,7 @@
     </row>
     <row r="14" spans="1:11" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="362" t="str">
-        <f>'Данные объект'!B17</f>
+        <f>IF('Данные объект'!B17="","",'Данные объект'!B17)</f>
       </c>
       <c r="B14" s="362"/>
       <c r="C14" s="362"/>
@@ -12167,7 +12167,7 @@
     </row>
     <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="362" t="str">
-        <f>'Данные объект'!B18</f>
+        <f>IF('Данные объект'!B18="","",'Данные объект'!B18)</f>
       </c>
       <c r="B15" s="362"/>
       <c r="C15" s="362"/>
@@ -12188,7 +12188,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="360" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="B17" s="360"/>
       <c r="C17" s="360"/>
@@ -12262,7 +12262,7 @@
       </c>
       <c r="B24" s="245"/>
       <c r="C24" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D24" s="247"/>
       <c r="E24" s="247"/>
@@ -12270,7 +12270,7 @@
       <c r="G24" s="6"/>
       <c r="H24" s="140"/>
       <c r="I24" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J24" s="247"/>
       <c r="K24" s="140"/>
@@ -12330,7 +12330,7 @@
       <c r="A28" s="245"/>
       <c r="B28" s="245"/>
       <c r="C28" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D28" s="247"/>
       <c r="E28" s="247"/>
@@ -12338,7 +12338,7 @@
       <c r="G28" s="6"/>
       <c r="H28" s="140"/>
       <c r="I28" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J28" s="247"/>
       <c r="K28" s="140"/>
@@ -12383,7 +12383,7 @@
       </c>
       <c r="B31" s="245"/>
       <c r="C31" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D31" s="247"/>
       <c r="E31" s="247"/>
@@ -12391,7 +12391,7 @@
       <c r="G31" s="6"/>
       <c r="H31" s="140"/>
       <c r="I31" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J31" s="247"/>
       <c r="K31" s="140"/>
@@ -12516,7 +12516,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A1" s="368" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="368"/>
       <c r="C1" s="368"/>
@@ -12527,7 +12527,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="369" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="369"/>
       <c r="J1" s="369"/>
@@ -12535,7 +12535,7 @@
     </row>
     <row r="2" spans="1:12" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="368" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="368"/>
       <c r="C2" s="368"/>
@@ -12563,7 +12563,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="371" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="371"/>
       <c r="J3" s="371"/>
@@ -12608,7 +12608,7 @@
       <c r="H6" s="176"/>
       <c r="I6" s="176"/>
       <c r="J6" s="374" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="374"/>
     </row>
@@ -13048,7 +13048,7 @@
       </c>
       <c r="B36" s="382"/>
       <c r="C36" s="390" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D36" s="390"/>
       <c r="E36" s="390"/>
@@ -13056,7 +13056,7 @@
       <c r="G36" s="195"/>
       <c r="H36" s="176"/>
       <c r="I36" s="390" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J36" s="390"/>
       <c r="K36" s="176"/>
@@ -13116,7 +13116,7 @@
       <c r="A40" s="382"/>
       <c r="B40" s="382"/>
       <c r="C40" s="390" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D40" s="390"/>
       <c r="E40" s="390"/>
@@ -13124,7 +13124,7 @@
       <c r="G40" s="195"/>
       <c r="H40" s="176"/>
       <c r="I40" s="390" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J40" s="390"/>
       <c r="K40" s="176"/>
@@ -13169,7 +13169,7 @@
       </c>
       <c r="B43" s="382"/>
       <c r="C43" s="390" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D43" s="390"/>
       <c r="E43" s="390"/>
@@ -13177,7 +13177,7 @@
       <c r="G43" s="195"/>
       <c r="H43" s="176"/>
       <c r="I43" s="390" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J43" s="390"/>
       <c r="K43" s="176"/>
@@ -13323,7 +13323,7 @@
       <c r="F5"/>
       <c r="G5"/>
     </row>
-    <row r="6" spans="1:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
         <v>188</v>
       </c>
@@ -13334,7 +13334,7 @@
       <c r="F6"/>
       <c r="G6"/>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
         <v>189</v>
       </c>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="B22" s="85"/>
       <c r="C22" s="43" t="str">
-        <f>CONCATENATE(B22," ",B23," ",B24)</f>
+        <f>IF(AND(B22="",B23="",B24=""),"",CONCATENATE(IF(B22="","",B22)," ",IF(B23="","",B23)," ",IF(B24="","",B24)))</f>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -13490,7 +13490,7 @@
         <v>200</v>
       </c>
       <c r="B23" s="85" t="str">
-        <f>'Данные организации'!B2</f>
+        <f>IF('Данные организации'!B2="","",'Данные организации'!B2)</f>
       </c>
       <c r="C23" s="43"/>
     </row>
@@ -13499,7 +13499,7 @@
         <v>187</v>
       </c>
       <c r="B24" s="85" t="str">
-        <f>'Данные организации'!B3</f>
+        <f>IF('Данные организации'!B3="","",'Данные организации'!B3)</f>
       </c>
       <c r="C24" s="43"/>
     </row>
@@ -13516,7 +13516,7 @@
       </c>
       <c r="B26" s="85"/>
       <c r="C26" s="43" t="str">
-        <f>CONCATENATE(B25," ",B22," ",B26)</f>
+        <f>IF(AND(B25="",B22="",B26=""),"",CONCATENATE(IF(B25="","",B25)," ",IF(B22="","",B22)," ",IF(B26="","",B26)))</f>
       </c>
     </row>
     <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="B27" s="85"/>
       <c r="C27" s="43" t="str">
-        <f>CONCATENATE(B27," ",B22)</f>
+        <f>IF(AND(B27="",B22=""),"",CONCATENATE(IF(B27="","",B27)," ",IF(B22="","",B22)))</f>
       </c>
     </row>
     <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13534,7 +13534,7 @@
       </c>
       <c r="B28" s="85"/>
       <c r="C28" s="44" t="str">
-        <f>CONCATENATE(B27," ",B22," ",B28)</f>
+        <f>IF(AND(B27="",B22="",B28=""),"",CONCATENATE(IF(B27="","",B27)," ",IF(B22="","",B22)," ",IF(B28="","",B28)))</f>
       </c>
     </row>
     <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="B29" s="85"/>
       <c r="C29" s="44" t="str">
-        <f>CONCATENATE(B27," ",B22," ",B28,".",B29)</f>
+        <f>IF(AND(B27="",B22="",B28="",B29=""),"",CONCATENATE(IF(B27="","",B27)," ",IF(B22="","",B22)," ",IF(B28="","",B28),".",IF(B29="","",B29)))</f>
       </c>
     </row>
     <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13552,7 +13552,7 @@
       </c>
       <c r="B30" s="85"/>
       <c r="C30" s="43" t="str">
-        <f>CONCATENATE(B30," ",B22)</f>
+        <f>IF(AND(B30="",B22=""),"",CONCATENATE(IF(B30="","",B30)," ",IF(B22="","",B22)))</f>
       </c>
     </row>
     <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13561,7 +13561,7 @@
       </c>
       <c r="B31" s="85"/>
       <c r="C31" s="44" t="str">
-        <f>CONCATENATE(B30," ",B22," ",B31)</f>
+        <f>IF(AND(B30="",B22="",B31=""),"",CONCATENATE(IF(B30="","",B30)," ",IF(B22="","",B22)," ",IF(B31="","",B31)))</f>
       </c>
     </row>
     <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="B32" s="85"/>
       <c r="C32" s="44" t="str">
-        <f>CONCATENATE(B30," ",B22," ",B31,".",B32)</f>
+        <f>IF(AND(B30="",B22="",B31="",B32=""),"",CONCATENATE(IF(B30="","",B30)," ",IF(B22="","",B22)," ",IF(B31="","",B31),".",IF(B32="","",B32)))</f>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -13584,7 +13584,7 @@
         <v>199</v>
       </c>
       <c r="B34" s="87" t="str">
-        <f>'Данные организации'!F1</f>
+        <f>IF('Данные организации'!F1="","",'Данные организации'!F1)</f>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -13592,7 +13592,7 @@
         <v>200</v>
       </c>
       <c r="B35" s="87" t="str">
-        <f>'Данные организации'!F2</f>
+        <f>IF('Данные организации'!F2="","",'Данные организации'!F2)</f>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -13600,7 +13600,7 @@
         <v>187</v>
       </c>
       <c r="B36" s="87" t="str">
-        <f>'Данные организации'!F3</f>
+        <f>IF('Данные организации'!F3="","",'Данные организации'!F3)</f>
       </c>
     </row>
     <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="B37" s="88"/>
       <c r="C37" s="36" t="str">
-        <f>CONCATENATE(B37," ",B34)</f>
+        <f>IF(AND(B37="",B34=""),"",CONCATENATE(IF(B37="","",B37)," ",IF(B34="","",B34)))</f>
       </c>
     </row>
     <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="B38" s="87"/>
       <c r="C38" s="36" t="str">
-        <f>CONCATENATE(B37," ",B34," ",B38)</f>
+        <f>IF(AND(B37="",B34="",B38=""),"",CONCATENATE(IF(B37="","",B37)," ",IF(B34="","",B34)," ",IF(B38="","",B38)))</f>
       </c>
     </row>
     <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="B39" s="87"/>
       <c r="C39" s="36" t="str">
-        <f>CONCATENATE(B39," ",B34)</f>
+        <f>IF(AND(B39="",B34=""),"",CONCATENATE(IF(B39="","",B39)," ",IF(B34="","",B34)))</f>
       </c>
     </row>
     <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13636,7 +13636,7 @@
       </c>
       <c r="B40" s="87"/>
       <c r="C40" s="36" t="str">
-        <f>CONCATENATE(B39," ",B34," ",B40)</f>
+        <f>IF(AND(B39="",B34="",B40=""),"",CONCATENATE(IF(B39="","",B39)," ",IF(B34="","",B34)," ",IF(B40="","",B40)))</f>
       </c>
     </row>
     <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13645,7 +13645,7 @@
       </c>
       <c r="B41" s="87"/>
       <c r="C41" s="36" t="str">
-        <f>CONCATENATE(B41," ",B34)</f>
+        <f>IF(AND(B41="",B34=""),"",CONCATENATE(IF(B41="","",B41)," ",IF(B34="","",B34)))</f>
       </c>
     </row>
     <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13654,7 +13654,7 @@
       </c>
       <c r="B42" s="87"/>
       <c r="C42" s="36" t="str">
-        <f>CONCATENATE(B41," ",B34," ",B42)</f>
+        <f>IF(AND(B41="",B34="",B42=""),"",CONCATENATE(IF(B41="","",B41)," ",IF(B34="","",B34)," ",IF(B42="","",B42)))</f>
       </c>
     </row>
     <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="B43" s="87"/>
       <c r="C43" s="36" t="str">
-        <f>CONCATENATE(B43," ",B34)</f>
+        <f>IF(AND(B43="",B34=""),"",CONCATENATE(IF(B43="","",B43)," ",IF(B34="","",B34)))</f>
       </c>
     </row>
     <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13672,7 +13672,7 @@
       </c>
       <c r="B44" s="87"/>
       <c r="C44" s="47" t="str">
-        <f>CONCATENATE(B43," ",B34," ",B44)</f>
+        <f>IF(AND(B43="",B34="",B44=""),"",CONCATENATE(IF(B43="","",B43)," ",IF(B34="","",B34)," ",IF(B44="","",B44)))</f>
       </c>
     </row>
     <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="B45" s="46"/>
       <c r="C45" s="36" t="str">
-        <f>CONCATENATE(B43," ",B34," ",B44,".",B45)</f>
+        <f>IF(AND(B43="",B34="",B44="",B45=""),"",CONCATENATE(IF(B43="","",B43)," ",IF(B34="","",B34)," ",IF(B44="","",B44),".",IF(B45="","",B45)))</f>
       </c>
     </row>
     <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13690,7 +13690,7 @@
       </c>
       <c r="B46" s="48"/>
       <c r="C46" s="36" t="str">
-        <f>CONCATENATE(B46," ",B34)</f>
+        <f>IF(AND(B46="",B34=""),"",CONCATENATE(IF(B46="","",B46)," ",IF(B34="","",B34)))</f>
       </c>
     </row>
     <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13699,7 +13699,7 @@
       </c>
       <c r="B47" s="48"/>
       <c r="C47" s="36" t="str">
-        <f>CONCATENATE(B46," ",B34," ",B47)</f>
+        <f>IF(AND(B46="",B34="",B47=""),"",CONCATENATE(IF(B46="","",B46)," ",IF(B34="","",B34)," ",IF(B47="","",B47)))</f>
       </c>
     </row>
     <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -13708,7 +13708,7 @@
       </c>
       <c r="B48" s="48"/>
       <c r="C48" s="36" t="str">
-        <f>CONCATENATE(B46," ",B34," ",B47,".",B48)</f>
+        <f>IF(AND(B46="",B34="",B47="",B48=""),"",CONCATENATE(IF(B46="","",B46)," ",IF(B34="","",B34)," ",IF(B47="","",B47),".",IF(B48="","",B48)))</f>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -13752,7 +13752,7 @@
         <v>208</v>
       </c>
       <c r="B55" s="86" t="str">
-        <f>$B$3</f>
+        <f>IF($B$3="","",$B$3)</f>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -13769,7 +13769,7 @@
       </c>
       <c r="B58" s="49"/>
       <c r="C58" s="36" t="str">
-        <f>CONCATENATE(A56," ",B60,", ",A63," ",B63)</f>
+        <f>IF(AND(A56="",B60="",A63="",B63=""),"",CONCATENATE(IF(A56="","",A56)," ",IF(B60="","",B60),", ",IF(A63="","",A63)," ",IF(B63="","",B63)))</f>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -13790,7 +13790,7 @@
       </c>
       <c r="B61" s="49"/>
       <c r="C61" s="36" t="str">
-        <f>CONCATENATE(B61," ",B58," ",B62)</f>
+        <f>IF(AND(B61="",B58="",B62=""),"",CONCATENATE(IF(B61="","",B61)," ",IF(B58="","",B58)," ",IF(B62="","",B62)))</f>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -14826,7 +14826,7 @@
     </row>
     <row r="5" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="235" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B5" s="235"/>
       <c r="C5" s="235"/>
@@ -14869,7 +14869,7 @@
     </row>
     <row r="11" spans="1:11" ht="22.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="233" t="str">
-        <f>'Данные объект'!B63</f>
+        <f>IF('Данные объект'!B63="","",'Данные объект'!B63)</f>
       </c>
       <c r="B11" s="233"/>
       <c r="C11" s="233"/>
@@ -14884,7 +14884,7 @@
     </row>
     <row r="12" spans="1:11" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="233" t="str">
-        <f>'Данные объект'!B68</f>
+        <f>IF('Данные объект'!B68="","",'Данные объект'!B68)</f>
       </c>
       <c r="B12" s="233"/>
       <c r="C12" s="233"/>
@@ -14899,7 +14899,7 @@
     </row>
     <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="229" t="str">
-        <f>'Данные объект'!C22</f>
+        <f>IF('Данные объект'!C22="","",'Данные объект'!C22)</f>
       </c>
       <c r="B13" s="229"/>
       <c r="C13" s="229"/>
@@ -14942,7 +14942,7 @@
     </row>
     <row r="21" spans="1:11" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="234" t="str">
-        <f>A5</f>
+        <f>IF(A5="","",A5)</f>
       </c>
       <c r="B21" s="234"/>
       <c r="C21" s="234"/>
@@ -14970,7 +14970,7 @@
     </row>
     <row r="23" spans="1:11" ht="22.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="234" t="str">
-        <f>'Данные объект'!B62</f>
+        <f>IF('Данные объект'!B62="","",'Данные объект'!B62)</f>
       </c>
       <c r="B23" s="234"/>
       <c r="C23" s="234"/>
@@ -15007,7 +15007,7 @@
       <c r="F29" s="227"/>
       <c r="G29" s="227"/>
       <c r="H29" s="228" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="I29" s="228"/>
       <c r="J29" s="150"/>
@@ -15030,7 +15030,7 @@
     </row>
     <row r="32" spans="1:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="231" t="str">
-        <f>'Данные объект'!B14</f>
+        <f>IF('Данные объект'!B14="","",'Данные объект'!B14)</f>
       </c>
       <c r="B32" s="231"/>
       <c r="C32" s="231"/>
@@ -15064,7 +15064,7 @@
       </c>
       <c r="B35" s="222"/>
       <c r="C35" s="225" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="D35" s="225"/>
       <c r="E35" s="225"/>
@@ -15094,7 +15094,7 @@
       </c>
       <c r="B37" s="222"/>
       <c r="C37" s="223" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="D37" s="223"/>
       <c r="E37" s="223"/>
@@ -15189,7 +15189,7 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F55" s="172" t="str">
-        <f>'Данные объект'!B9</f>
+        <f>IF('Данные объект'!B9="","",'Данные объект'!B9)</f>
       </c>
     </row>
   </sheetData>
@@ -15247,7 +15247,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -15256,7 +15256,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -15264,7 +15264,7 @@
     </row>
     <row r="2" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -15288,7 +15288,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -15319,7 +15319,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -15593,7 +15593,7 @@
         <v>270</v>
       </c>
       <c r="C26" s="168">
-        <f>'Данные объект'!B10</f>
+        <f>IF('Данные объект'!B10="","",'Данные объект'!B10)</f>
       </c>
       <c r="D26" s="3" t="s">
         <v>265</v>
@@ -15605,7 +15605,7 @@
       </c>
       <c r="B27" s="245"/>
       <c r="C27" s="168">
-        <f>'Данные объект'!B11</f>
+        <f>IF('Данные объект'!B11="","",'Данные объект'!B11)</f>
       </c>
       <c r="D27" s="3" t="s">
         <v>267</v>
@@ -15616,7 +15616,7 @@
         <v>272</v>
       </c>
       <c r="C28" s="168" t="str">
-        <f>'Данные объект'!B12</f>
+        <f>IF('Данные объект'!B12="","",'Данные объект'!B12)</f>
       </c>
       <c r="D28" s="3" t="s">
         <v>269</v>
@@ -15720,10 +15720,10 @@
         <v>45</v>
       </c>
       <c r="I34" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J34" s="265" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K34" s="265"/>
     </row>
@@ -15743,10 +15743,10 @@
       </c>
       <c r="H35" s="142"/>
       <c r="I35" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J35" s="240" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K35" s="240"/>
     </row>
@@ -15766,10 +15766,10 @@
       </c>
       <c r="H36" s="142"/>
       <c r="I36" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J36" s="240" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K36" s="240"/>
     </row>
@@ -15789,10 +15789,10 @@
       </c>
       <c r="H37" s="142"/>
       <c r="I37" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J37" s="240" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K37" s="240"/>
     </row>
@@ -15822,13 +15822,13 @@
       </c>
       <c r="B40" s="245"/>
       <c r="C40" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D40" s="247"/>
       <c r="E40" s="247"/>
       <c r="G40" s="6"/>
       <c r="I40" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J40" s="247"/>
     </row>
@@ -15885,13 +15885,13 @@
       <c r="A44" s="245"/>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
       <c r="G44" s="6"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J44" s="247"/>
     </row>
@@ -15920,13 +15920,13 @@
       </c>
       <c r="B47" s="245"/>
       <c r="C47" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D47" s="247"/>
       <c r="E47" s="247"/>
       <c r="G47" s="6"/>
       <c r="I47" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J47" s="247"/>
     </row>
@@ -19170,7 +19170,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -19179,7 +19179,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -19187,7 +19187,7 @@
     </row>
     <row r="2" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -19211,7 +19211,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -19242,7 +19242,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -19412,7 +19412,7 @@
         <v>264</v>
       </c>
       <c r="C17" s="3">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D17" s="3" t="s">
         <v>265</v>
@@ -19423,7 +19423,7 @@
         <v>266</v>
       </c>
       <c r="C18" s="3">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D18" s="3" t="s">
         <v>267</v>
@@ -19434,7 +19434,7 @@
         <v>268</v>
       </c>
       <c r="C19" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D19" s="3" t="s">
         <v>269</v>
@@ -19537,10 +19537,10 @@
         <v>45</v>
       </c>
       <c r="I25" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J25" s="290" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K25" s="291"/>
     </row>
@@ -19560,10 +19560,10 @@
       </c>
       <c r="H26" s="199"/>
       <c r="I26" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J26" s="292" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K26" s="293"/>
     </row>
@@ -19583,10 +19583,10 @@
       </c>
       <c r="H27" s="199"/>
       <c r="I27" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J27" s="292" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K27" s="293"/>
     </row>
@@ -19606,10 +19606,10 @@
       </c>
       <c r="H28" s="199"/>
       <c r="I28" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J28" s="292" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K28" s="293"/>
     </row>
@@ -19700,7 +19700,7 @@
       </c>
       <c r="B37" s="245"/>
       <c r="C37" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D37" s="247"/>
       <c r="E37" s="247"/>
@@ -19708,7 +19708,7 @@
       <c r="G37" s="6"/>
       <c r="H37" s="140"/>
       <c r="I37" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J37" s="247"/>
       <c r="K37" s="140"/>
@@ -19768,7 +19768,7 @@
       <c r="A41" s="245"/>
       <c r="B41" s="245"/>
       <c r="C41" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D41" s="247"/>
       <c r="E41" s="247"/>
@@ -19776,7 +19776,7 @@
       <c r="G41" s="6"/>
       <c r="H41" s="140"/>
       <c r="I41" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J41" s="247"/>
       <c r="K41" s="140"/>
@@ -19821,7 +19821,7 @@
       </c>
       <c r="B44" s="245"/>
       <c r="C44" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D44" s="247"/>
       <c r="E44" s="247"/>
@@ -19829,7 +19829,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="140"/>
       <c r="I44" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J44" s="247"/>
       <c r="K44" s="140"/>
@@ -19951,7 +19951,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -19960,7 +19960,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -19968,7 +19968,7 @@
     </row>
     <row r="2" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -19992,7 +19992,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -20023,7 +20023,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -20370,10 +20370,10 @@
         <v>45</v>
       </c>
       <c r="I33" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J33" s="265" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K33" s="265"/>
     </row>
@@ -20393,10 +20393,10 @@
       </c>
       <c r="H34" s="142"/>
       <c r="I34" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J34" s="240" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K34" s="240"/>
     </row>
@@ -20416,10 +20416,10 @@
       </c>
       <c r="H35" s="142"/>
       <c r="I35" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J35" s="240" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K35" s="240"/>
     </row>
@@ -20439,10 +20439,10 @@
       </c>
       <c r="H36" s="142"/>
       <c r="I36" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J36" s="240" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K36" s="240"/>
     </row>
@@ -20452,7 +20452,7 @@
       </c>
       <c r="B38" s="245"/>
       <c r="C38" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D38" s="247"/>
       <c r="E38" s="247"/>
@@ -20460,7 +20460,7 @@
       <c r="G38" s="6"/>
       <c r="H38" s="140"/>
       <c r="I38" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J38" s="247"/>
       <c r="K38" s="140"/>
@@ -20520,7 +20520,7 @@
       <c r="A42" s="245"/>
       <c r="B42" s="245"/>
       <c r="C42" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D42" s="247"/>
       <c r="E42" s="247"/>
@@ -20528,7 +20528,7 @@
       <c r="G42" s="6"/>
       <c r="H42" s="140"/>
       <c r="I42" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J42" s="247"/>
       <c r="K42" s="140"/>
@@ -20573,7 +20573,7 @@
       </c>
       <c r="B45" s="245"/>
       <c r="C45" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D45" s="247"/>
       <c r="E45" s="247"/>
@@ -20581,7 +20581,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="140"/>
       <c r="I45" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J45" s="247"/>
       <c r="K45" s="140"/>
@@ -20686,7 +20686,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -20695,7 +20695,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -20703,7 +20703,7 @@
     </row>
     <row r="2" spans="1:11" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -20727,7 +20727,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -21352,10 +21352,10 @@
         <v>45</v>
       </c>
       <c r="I48" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J48" s="265" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K48" s="265"/>
     </row>
@@ -21375,10 +21375,10 @@
       </c>
       <c r="H49" s="142"/>
       <c r="I49" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J49" s="240" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K49" s="240"/>
     </row>
@@ -21398,10 +21398,10 @@
       </c>
       <c r="H50" s="142"/>
       <c r="I50" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J50" s="240" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K50" s="240"/>
     </row>
@@ -21421,10 +21421,10 @@
       </c>
       <c r="H51" s="142"/>
       <c r="I51" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J51" s="240" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K51" s="240"/>
     </row>
@@ -21449,7 +21449,7 @@
       </c>
       <c r="B56" s="245"/>
       <c r="C56" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D56" s="247"/>
       <c r="E56" s="247"/>
@@ -21457,7 +21457,7 @@
       <c r="G56" s="6"/>
       <c r="H56" s="140"/>
       <c r="I56" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J56" s="247"/>
       <c r="K56" s="140"/>
@@ -21517,7 +21517,7 @@
       <c r="A60" s="245"/>
       <c r="B60" s="245"/>
       <c r="C60" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D60" s="247"/>
       <c r="E60" s="247"/>
@@ -21525,7 +21525,7 @@
       <c r="G60" s="6"/>
       <c r="H60" s="140"/>
       <c r="I60" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J60" s="247"/>
       <c r="K60" s="140"/>
@@ -21570,7 +21570,7 @@
       </c>
       <c r="B63" s="245"/>
       <c r="C63" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D63" s="247"/>
       <c r="E63" s="247"/>
@@ -21578,7 +21578,7 @@
       <c r="G63" s="6"/>
       <c r="H63" s="140"/>
       <c r="I63" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J63" s="247"/>
       <c r="K63" s="140"/>
@@ -21707,7 +21707,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="262" t="str">
-        <f>'Данные объект'!B58</f>
+        <f>IF('Данные объект'!B58="","",'Данные объект'!B58)</f>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -21716,7 +21716,7 @@
         <v>11</v>
       </c>
       <c r="H1" s="259" t="str">
-        <f>'Данные объект'!B34</f>
+        <f>IF('Данные объект'!B34="","",'Данные объект'!B34)</f>
       </c>
       <c r="I1" s="259"/>
       <c r="J1" s="259"/>
@@ -21724,7 +21724,7 @@
     </row>
     <row r="2" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="262" t="str">
-        <f>'Данные объект'!C58</f>
+        <f>IF('Данные объект'!C58="","",'Данные объект'!C58)</f>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -21748,7 +21748,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="261" t="str">
-        <f>'Данные объект'!B5</f>
+        <f>IF('Данные объект'!B5="","",'Данные объект'!B5)</f>
       </c>
       <c r="I3" s="261"/>
       <c r="J3" s="261"/>
@@ -21779,7 +21779,7 @@
       <c r="B6" s="250"/>
       <c r="C6" s="250"/>
       <c r="J6" s="263" t="str">
-        <f>'Данные объект'!B8</f>
+        <f>IF('Данные объект'!B8="","",'Данные объект'!B8)</f>
       </c>
       <c r="K6" s="263"/>
     </row>
@@ -22059,10 +22059,10 @@
         <v>45</v>
       </c>
       <c r="I27" s="158">
-        <f>Оборудование!I4</f>
+        <f>IF(Оборудование!I4="","",Оборудование!I4)</f>
       </c>
       <c r="J27" s="265" t="str">
-        <f>Оборудование!J4</f>
+        <f>IF(Оборудование!J4="","",Оборудование!J4)</f>
       </c>
       <c r="K27" s="265"/>
     </row>
@@ -22082,10 +22082,10 @@
       </c>
       <c r="H28" s="142"/>
       <c r="I28" s="158">
-        <f>Оборудование!I3</f>
+        <f>IF(Оборудование!I3="","",Оборудование!I3)</f>
       </c>
       <c r="J28" s="240" t="str">
-        <f>Оборудование!J3</f>
+        <f>IF(Оборудование!J3="","",Оборудование!J3)</f>
       </c>
       <c r="K28" s="240"/>
     </row>
@@ -22105,10 +22105,10 @@
       </c>
       <c r="H29" s="142"/>
       <c r="I29" s="158">
-        <f>Оборудование!I12</f>
+        <f>IF(Оборудование!I12="","",Оборудование!I12)</f>
       </c>
       <c r="J29" s="240" t="str">
-        <f>Оборудование!J12</f>
+        <f>IF(Оборудование!J12="","",Оборудование!J12)</f>
       </c>
       <c r="K29" s="240"/>
     </row>
@@ -22128,10 +22128,10 @@
       </c>
       <c r="H30" s="142"/>
       <c r="I30" s="158">
-        <f>Оборудование!I13</f>
+        <f>IF(Оборудование!I13="","",Оборудование!I13)</f>
       </c>
       <c r="J30" s="240" t="str">
-        <f>Оборудование!J13</f>
+        <f>IF(Оборудование!J13="","",Оборудование!J13)</f>
       </c>
       <c r="K30" s="240"/>
     </row>
@@ -22155,7 +22155,7 @@
         <v>274</v>
       </c>
       <c r="C32" s="392">
-        <f>прот.№1!C26</f>
+        <f>IF(прот.№1!C26="","",прот.№1!C26)</f>
       </c>
       <c r="D32" s="3" t="s">
         <v>265</v>
@@ -22166,7 +22166,7 @@
         <v>275</v>
       </c>
       <c r="C33" s="392">
-        <f>прот.№1!C27</f>
+        <f>IF(прот.№1!C27="","",прот.№1!C27)</f>
       </c>
       <c r="D33" s="3" t="s">
         <v>267</v>
@@ -22177,7 +22177,7 @@
         <v>276</v>
       </c>
       <c r="C34" s="392" t="str">
-        <f>прот.№1!C28</f>
+        <f>IF(прот.№1!C28="","",прот.№1!C28)</f>
       </c>
       <c r="D34" s="3" t="s">
         <v>269</v>
@@ -22222,7 +22222,7 @@
       </c>
       <c r="B41" s="245"/>
       <c r="C41" s="247" t="str">
-        <f>'Данные объект'!$B$64</f>
+        <f>IF('Данные объект'!$B$64="","",'Данные объект'!$B$64)</f>
       </c>
       <c r="D41" s="247"/>
       <c r="E41" s="247"/>
@@ -22230,7 +22230,7 @@
       <c r="G41" s="6"/>
       <c r="H41" s="140"/>
       <c r="I41" s="247" t="str">
-        <f>'Данные объект'!$B$65</f>
+        <f>IF('Данные объект'!$B$65="","",'Данные объект'!$B$65)</f>
       </c>
       <c r="J41" s="247"/>
       <c r="K41" s="140"/>
@@ -22290,7 +22290,7 @@
       <c r="A45" s="245"/>
       <c r="B45" s="245"/>
       <c r="C45" s="247" t="str">
-        <f>'Данные объект'!$B$66</f>
+        <f>IF('Данные объект'!$B$66="","",'Данные объект'!$B$66)</f>
       </c>
       <c r="D45" s="247"/>
       <c r="E45" s="247"/>
@@ -22298,7 +22298,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="140"/>
       <c r="I45" s="247" t="str">
-        <f>'Данные объект'!$B$67</f>
+        <f>IF('Данные объект'!$B$67="","",'Данные объект'!$B$67)</f>
       </c>
       <c r="J45" s="247"/>
       <c r="K45" s="140"/>
@@ -22343,7 +22343,7 @@
       </c>
       <c r="B48" s="245"/>
       <c r="C48" s="247" t="str">
-        <f>'Данные объект'!$B$61</f>
+        <f>IF('Данные объект'!$B$61="","",'Данные объект'!$B$61)</f>
       </c>
       <c r="D48" s="247"/>
       <c r="E48" s="247"/>
@@ -22351,7 +22351,7 @@
       <c r="G48" s="6"/>
       <c r="H48" s="140"/>
       <c r="I48" s="247" t="str">
-        <f>'Данные объект'!$B$62</f>
+        <f>IF('Данные объект'!$B$62="","",'Данные объект'!$B$62)</f>
       </c>
       <c r="J48" s="247"/>
       <c r="K48" s="140"/>

</xml_diff>